<commit_message>
Guard Vatinterface month links across all packages and republish Ltd VAT workbooks
No test walked the shipped workbooks' month links: reconciliation reads
no VAT cell (ltd CELL_MAP has none), the roundtrip test only runs the
template year-end where the month rewrite is a no-op, and the dropdown
guard checks the date chain but not the D/F/H/J/M money columns. The
new guard walks every packages Vatreturns.xlsx and Vat.xlsx and asserts
each month row reads its own month tab from Sales/Purchases and that
the sibling workbooks name their tabs in the same sequence. Against the
old packages it reported 1620 wrong-tab links.

Regenerate the 90 Ltd Vatreturns.xlsx with the fixed pipeline so the
shipped packages match; only Vatreturns.xlsx differs per package.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012mDxaoTv97DNa41DXrsLWu
</commit_message>
<xml_diff>
--- a/packages/GB Accounts Company 2020-04-30 (Apr20) Excel 2007/Vatreturns.xlsx
+++ b/packages/GB Accounts Company 2020-04-30 (Apr20) Excel 2007/Vatreturns.xlsx
@@ -16405,7 +16405,7 @@
       </c>
       <c r="L8" s="115"/>
       <c r="M8" s="116">
-        <f>IF([2]Oct!$G$4&gt;0,[2]Oct!$G$4,0)</f>
+        <f>IF([2]Jul!$G$4&gt;0,[2]Jul!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N8" s="57"/>
@@ -16454,7 +16454,7 @@
       </c>
       <c r="L9" s="115"/>
       <c r="M9" s="116">
-        <f>IF([2]Jun!$G$4&gt;0,[2]Jun!$G$4,0)</f>
+        <f>IF([2]Aug!$G$4&gt;0,[2]Aug!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N9" s="57"/>
@@ -16503,7 +16503,7 @@
       </c>
       <c r="L10" s="115"/>
       <c r="M10" s="116">
-        <f>IF([2]Apr!$G$4&gt;0,[2]Apr!$G$4,0)</f>
+        <f>IF([2]Sep!$G$4&gt;0,[2]Sep!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N10" s="57"/>
@@ -16552,7 +16552,7 @@
       </c>
       <c r="L11" s="115"/>
       <c r="M11" s="116">
-        <f>IF([2]Jul!$G$4&gt;0,[2]Jul!$G$4,0)</f>
+        <f>IF([2]Oct!$G$4&gt;0,[2]Oct!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N11" s="57"/>
@@ -16601,7 +16601,7 @@
       </c>
       <c r="L12" s="115"/>
       <c r="M12" s="116">
-        <f>IF([2]Dec!$G$4&gt;0,[2]Dec!$G$4,0)</f>
+        <f>IF([2]Nov!$G$4&gt;0,[2]Nov!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N12" s="57"/>
@@ -16650,7 +16650,7 @@
       </c>
       <c r="L13" s="115"/>
       <c r="M13" s="116">
-        <f>IF([2]Sep!$G$4&gt;0,[2]Sep!$G$4,0)</f>
+        <f>IF([2]Dec!$G$4&gt;0,[2]Dec!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N13" s="57"/>
@@ -16699,7 +16699,7 @@
       </c>
       <c r="L14" s="115"/>
       <c r="M14" s="116">
-        <f>IF([2]Sep!$G$4&gt;0,[2]Sep!$G$4,0)</f>
+        <f>IF([2]Jan!$G$4&gt;0,[2]Jan!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N14" s="57"/>
@@ -16748,7 +16748,7 @@
       </c>
       <c r="L15" s="115"/>
       <c r="M15" s="116">
-        <f>IF([2]Dec!$G$4&gt;0,[2]Dec!$G$4,0)</f>
+        <f>IF([2]Feb!$G$4&gt;0,[2]Feb!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N15" s="57"/>
@@ -16797,7 +16797,7 @@
       </c>
       <c r="L16" s="115"/>
       <c r="M16" s="116">
-        <f>IF([2]Jul!$G$4&gt;0,[2]Jul!$G$4,0)</f>
+        <f>IF([2]Mar!$G$4&gt;0,[2]Mar!$G$4,0)</f>
         <v>0</v>
       </c>
       <c r="N16" s="57"/>

</xml_diff>